<commit_message>
feat(luban): add crop config table and seed/produce items
Co-authored-by: Cursor <cursoragent@cursor.com>
</commit_message>
<xml_diff>
--- a/Tools/Luban/DataTables/Datas/CozyYard/item.xlsx
+++ b/Tools/Luban/DataTables/Datas/CozyYard/item.xlsx
@@ -432,7 +432,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F5"/>
+  <dimension ref="A1:F15"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="9" customWidth="1" min="1" max="1"/>
@@ -579,6 +579,246 @@
         </is>
       </c>
     </row>
+    <row r="6">
+      <c r="A6" t="inlineStr"/>
+      <c r="B6" t="n">
+        <v>2001</v>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>白菜种子</t>
+        </is>
+      </c>
+      <c r="D6" t="inlineStr">
+        <is>
+          <t>Seed</t>
+        </is>
+      </c>
+      <c r="E6" t="n">
+        <v>50</v>
+      </c>
+      <c r="F6" t="inlineStr">
+        <is>
+          <t>种植白菜</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr"/>
+      <c r="B7" t="n">
+        <v>2002</v>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>萝卜种子</t>
+        </is>
+      </c>
+      <c r="D7" t="inlineStr">
+        <is>
+          <t>Seed</t>
+        </is>
+      </c>
+      <c r="E7" t="n">
+        <v>50</v>
+      </c>
+      <c r="F7" t="inlineStr">
+        <is>
+          <t>种植萝卜</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr"/>
+      <c r="B8" t="n">
+        <v>2003</v>
+      </c>
+      <c r="C8" t="inlineStr">
+        <is>
+          <t>糯米种子</t>
+        </is>
+      </c>
+      <c r="D8" t="inlineStr">
+        <is>
+          <t>Seed</t>
+        </is>
+      </c>
+      <c r="E8" t="n">
+        <v>50</v>
+      </c>
+      <c r="F8" t="inlineStr">
+        <is>
+          <t>种植糯米</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr"/>
+      <c r="B9" t="n">
+        <v>2004</v>
+      </c>
+      <c r="C9" t="inlineStr">
+        <is>
+          <t>菊花种子</t>
+        </is>
+      </c>
+      <c r="D9" t="inlineStr">
+        <is>
+          <t>Seed</t>
+        </is>
+      </c>
+      <c r="E9" t="n">
+        <v>50</v>
+      </c>
+      <c r="F9" t="inlineStr">
+        <is>
+          <t>种植菊花</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr"/>
+      <c r="B10" t="n">
+        <v>2005</v>
+      </c>
+      <c r="C10" t="inlineStr">
+        <is>
+          <t>辣椒种子</t>
+        </is>
+      </c>
+      <c r="D10" t="inlineStr">
+        <is>
+          <t>Seed</t>
+        </is>
+      </c>
+      <c r="E10" t="n">
+        <v>50</v>
+      </c>
+      <c r="F10" t="inlineStr">
+        <is>
+          <t>种植辣椒</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr"/>
+      <c r="B11" t="n">
+        <v>3001</v>
+      </c>
+      <c r="C11" t="inlineStr">
+        <is>
+          <t>白菜</t>
+        </is>
+      </c>
+      <c r="D11" t="inlineStr">
+        <is>
+          <t>Product</t>
+        </is>
+      </c>
+      <c r="E11" t="n">
+        <v>50</v>
+      </c>
+      <c r="F11" t="inlineStr">
+        <is>
+          <t>新鲜白菜</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr"/>
+      <c r="B12" t="n">
+        <v>3002</v>
+      </c>
+      <c r="C12" t="inlineStr">
+        <is>
+          <t>萝卜</t>
+        </is>
+      </c>
+      <c r="D12" t="inlineStr">
+        <is>
+          <t>Product</t>
+        </is>
+      </c>
+      <c r="E12" t="n">
+        <v>50</v>
+      </c>
+      <c r="F12" t="inlineStr">
+        <is>
+          <t>新鲜萝卜</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr"/>
+      <c r="B13" t="n">
+        <v>3003</v>
+      </c>
+      <c r="C13" t="inlineStr">
+        <is>
+          <t>糯米</t>
+        </is>
+      </c>
+      <c r="D13" t="inlineStr">
+        <is>
+          <t>Product</t>
+        </is>
+      </c>
+      <c r="E13" t="n">
+        <v>50</v>
+      </c>
+      <c r="F13" t="inlineStr">
+        <is>
+          <t>饱满的糯米</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr"/>
+      <c r="B14" t="n">
+        <v>3004</v>
+      </c>
+      <c r="C14" t="inlineStr">
+        <is>
+          <t>菊花</t>
+        </is>
+      </c>
+      <c r="D14" t="inlineStr">
+        <is>
+          <t>Product</t>
+        </is>
+      </c>
+      <c r="E14" t="n">
+        <v>50</v>
+      </c>
+      <c r="F14" t="inlineStr">
+        <is>
+          <t>新鲜菊花</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr"/>
+      <c r="B15" t="n">
+        <v>3005</v>
+      </c>
+      <c r="C15" t="inlineStr">
+        <is>
+          <t>辣椒</t>
+        </is>
+      </c>
+      <c r="D15" t="inlineStr">
+        <is>
+          <t>Product</t>
+        </is>
+      </c>
+      <c r="E15" t="n">
+        <v>50</v>
+      </c>
+      <c r="F15" t="inlineStr">
+        <is>
+          <t>新鲜辣椒</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
feat(luban): add animal config table and egg produce item
Co-authored-by: Cursor <cursoragent@cursor.com>
</commit_message>
<xml_diff>
--- a/Tools/Luban/DataTables/Datas/CozyYard/item.xlsx
+++ b/Tools/Luban/DataTables/Datas/CozyYard/item.xlsx
@@ -432,7 +432,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F15"/>
+  <dimension ref="A1:F16"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="9" customWidth="1" min="1" max="1"/>
@@ -819,6 +819,30 @@
         </is>
       </c>
     </row>
+    <row r="16">
+      <c r="A16" t="inlineStr"/>
+      <c r="B16" t="n">
+        <v>3101</v>
+      </c>
+      <c r="C16" t="inlineStr">
+        <is>
+          <t>鸡蛋</t>
+        </is>
+      </c>
+      <c r="D16" t="inlineStr">
+        <is>
+          <t>Product</t>
+        </is>
+      </c>
+      <c r="E16" t="n">
+        <v>50</v>
+      </c>
+      <c r="F16" t="inlineStr">
+        <is>
+          <t>新鲜鸡蛋</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
feat(luban): add recipe table and craft-related items
Add recipe config with 9 crafting recipes and extend item table with
intermediate materials, final products, tree produce, and junk item.

Co-authored-by: Cursor <cursoragent@cursor.com>
</commit_message>
<xml_diff>
--- a/Tools/Luban/DataTables/Datas/CozyYard/item.xlsx
+++ b/Tools/Luban/DataTables/Datas/CozyYard/item.xlsx
@@ -432,7 +432,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F16"/>
+  <dimension ref="A1:F28"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="9" customWidth="1" min="1" max="1"/>
@@ -440,7 +440,7 @@
     <col width="16" customWidth="1" min="3" max="3"/>
     <col width="12" customWidth="1" min="4" max="4"/>
     <col width="16" customWidth="1" min="5" max="5"/>
-    <col width="22" customWidth="1" min="6" max="6"/>
+    <col width="25" customWidth="1" min="6" max="6"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -843,6 +843,294 @@
         </is>
       </c>
     </row>
+    <row r="17">
+      <c r="A17" t="inlineStr"/>
+      <c r="B17" t="n">
+        <v>3006</v>
+      </c>
+      <c r="C17" t="inlineStr">
+        <is>
+          <t>桂花</t>
+        </is>
+      </c>
+      <c r="D17" t="inlineStr">
+        <is>
+          <t>Product</t>
+        </is>
+      </c>
+      <c r="E17" t="n">
+        <v>50</v>
+      </c>
+      <c r="F17" t="inlineStr">
+        <is>
+          <t>秋天采集</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="inlineStr"/>
+      <c r="B18" t="n">
+        <v>3007</v>
+      </c>
+      <c r="C18" t="inlineStr">
+        <is>
+          <t>柿子</t>
+        </is>
+      </c>
+      <c r="D18" t="inlineStr">
+        <is>
+          <t>Product</t>
+        </is>
+      </c>
+      <c r="E18" t="n">
+        <v>50</v>
+      </c>
+      <c r="F18" t="inlineStr">
+        <is>
+          <t>秋天采集</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="inlineStr"/>
+      <c r="B19" t="n">
+        <v>4001</v>
+      </c>
+      <c r="C19" t="inlineStr">
+        <is>
+          <t>桂花干</t>
+        </is>
+      </c>
+      <c r="D19" t="inlineStr">
+        <is>
+          <t>Material</t>
+        </is>
+      </c>
+      <c r="E19" t="n">
+        <v>50</v>
+      </c>
+      <c r="F19" t="inlineStr">
+        <is>
+          <t>晾晒桂花制得</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="inlineStr"/>
+      <c r="B20" t="n">
+        <v>4002</v>
+      </c>
+      <c r="C20" t="inlineStr">
+        <is>
+          <t>糯米粉</t>
+        </is>
+      </c>
+      <c r="D20" t="inlineStr">
+        <is>
+          <t>Material</t>
+        </is>
+      </c>
+      <c r="E20" t="n">
+        <v>50</v>
+      </c>
+      <c r="F20" t="inlineStr">
+        <is>
+          <t>石磨糯米制得</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="inlineStr"/>
+      <c r="B21" t="n">
+        <v>4003</v>
+      </c>
+      <c r="C21" t="inlineStr">
+        <is>
+          <t>萝卜干</t>
+        </is>
+      </c>
+      <c r="D21" t="inlineStr">
+        <is>
+          <t>Material</t>
+        </is>
+      </c>
+      <c r="E21" t="n">
+        <v>50</v>
+      </c>
+      <c r="F21" t="inlineStr">
+        <is>
+          <t>晾晒萝卜制得</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" t="inlineStr"/>
+      <c r="B22" t="n">
+        <v>4004</v>
+      </c>
+      <c r="C22" t="inlineStr">
+        <is>
+          <t>菊花干</t>
+        </is>
+      </c>
+      <c r="D22" t="inlineStr">
+        <is>
+          <t>Material</t>
+        </is>
+      </c>
+      <c r="E22" t="n">
+        <v>50</v>
+      </c>
+      <c r="F22" t="inlineStr">
+        <is>
+          <t>晾晒菊花制得</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" t="inlineStr"/>
+      <c r="B23" t="n">
+        <v>5001</v>
+      </c>
+      <c r="C23" t="inlineStr">
+        <is>
+          <t>桂花糕</t>
+        </is>
+      </c>
+      <c r="D23" t="inlineStr">
+        <is>
+          <t>Product</t>
+        </is>
+      </c>
+      <c r="E23" t="n">
+        <v>20</v>
+      </c>
+      <c r="F23" t="inlineStr">
+        <is>
+          <t>香甜的桂花糕</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" t="inlineStr"/>
+      <c r="B24" t="n">
+        <v>5002</v>
+      </c>
+      <c r="C24" t="inlineStr">
+        <is>
+          <t>辣炒蛋</t>
+        </is>
+      </c>
+      <c r="D24" t="inlineStr">
+        <is>
+          <t>Product</t>
+        </is>
+      </c>
+      <c r="E24" t="n">
+        <v>20</v>
+      </c>
+      <c r="F24" t="inlineStr">
+        <is>
+          <t>简单美味</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" t="inlineStr"/>
+      <c r="B25" t="n">
+        <v>5003</v>
+      </c>
+      <c r="C25" t="inlineStr">
+        <is>
+          <t>清炒白菜</t>
+        </is>
+      </c>
+      <c r="D25" t="inlineStr">
+        <is>
+          <t>Product</t>
+        </is>
+      </c>
+      <c r="E25" t="n">
+        <v>20</v>
+      </c>
+      <c r="F25" t="inlineStr">
+        <is>
+          <t>清淡爽口</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" t="inlineStr"/>
+      <c r="B26" t="n">
+        <v>5004</v>
+      </c>
+      <c r="C26" t="inlineStr">
+        <is>
+          <t>菊花茶</t>
+        </is>
+      </c>
+      <c r="D26" t="inlineStr">
+        <is>
+          <t>Product</t>
+        </is>
+      </c>
+      <c r="E26" t="n">
+        <v>20</v>
+      </c>
+      <c r="F26" t="inlineStr">
+        <is>
+          <t>清香提神</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" t="inlineStr"/>
+      <c r="B27" t="n">
+        <v>5005</v>
+      </c>
+      <c r="C27" t="inlineStr">
+        <is>
+          <t>柿饼</t>
+        </is>
+      </c>
+      <c r="D27" t="inlineStr">
+        <is>
+          <t>Product</t>
+        </is>
+      </c>
+      <c r="E27" t="n">
+        <v>20</v>
+      </c>
+      <c r="F27" t="inlineStr">
+        <is>
+          <t>甜糯柿饼</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" t="inlineStr"/>
+      <c r="B28" t="n">
+        <v>9001</v>
+      </c>
+      <c r="C28" t="inlineStr">
+        <is>
+          <t>黑暗料理</t>
+        </is>
+      </c>
+      <c r="D28" t="inlineStr">
+        <is>
+          <t>Material</t>
+        </is>
+      </c>
+      <c r="E28" t="n">
+        <v>10</v>
+      </c>
+      <c r="F28" t="inlineStr">
+        <is>
+          <t>实验失败的产物</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>